<commit_message>
ingesta: snapshot 2026-07-17 18:33 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-17/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-17/CORDOBA_JUL26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448DCEAF-AC30-4CFF-8B38-FB472E8870E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FB4634-3BE0-4265-A2AF-A6685D3CD2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
   <sheets>
     <sheet name="ENERO_2026" sheetId="1" r:id="rId1"/>
@@ -238,7 +238,7 @@
     <numFmt numFmtId="168" formatCode="_ [$€]\ * #,##0.00_ ;_ [$€]\ * \-#,##0.00_ ;_ [$€]\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="169" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="39" x14ac:knownFonts="1">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10005,7 +10005,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>-1</c:v>
@@ -13001,17 +13001,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B573599A-0B73-477B-832F-8EC63503F52D}">
   <dimension ref="A2:AK17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="5" max="35" width="5.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.25" customWidth="1"/>
+    <col min="3" max="3" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.25" customWidth="1"/>
+    <col min="5" max="35" width="5.875" customWidth="1"/>
     <col min="36" max="36" width="16" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" ht="15.75">
       <c r="A2" s="17" t="s">
         <v>26</v>
       </c>
@@ -13124,7 +13124,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" ht="15.75">
       <c r="A3" s="1">
         <v>13035501</v>
       </c>
@@ -13238,7 +13238,7 @@
         <v>8.046153846153846</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" ht="15.75">
       <c r="A4" s="1">
         <v>25025170</v>
       </c>
@@ -13352,7 +13352,7 @@
         <v>15.358620689655174</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" ht="15.75">
       <c r="A5" s="1">
         <v>25020140</v>
       </c>
@@ -13466,7 +13466,7 @@
         <v>15.933333333333334</v>
       </c>
     </row>
-    <row r="6" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="15.75">
       <c r="A6" s="1">
         <v>25025160</v>
       </c>
@@ -13580,7 +13580,7 @@
         <v>19.965384615384615</v>
       </c>
     </row>
-    <row r="7" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="15.75">
       <c r="A7" s="1">
         <v>25025190</v>
       </c>
@@ -13694,7 +13694,7 @@
         <v>20.685185185185187</v>
       </c>
     </row>
-    <row r="8" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="15.75">
       <c r="A8" s="1">
         <v>25020470</v>
       </c>
@@ -13808,7 +13808,7 @@
         <v>19.631034482758619</v>
       </c>
     </row>
-    <row r="9" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="15.75">
       <c r="A9" s="1">
         <v>25020700</v>
       </c>
@@ -13922,7 +13922,7 @@
         <v>15.135714285714288</v>
       </c>
     </row>
-    <row r="10" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="15.75">
       <c r="A10" s="1">
         <v>13015040</v>
       </c>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="AK10" s="8"/>
     </row>
-    <row r="11" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="15.75">
       <c r="A11" s="1">
         <v>13085010</v>
       </c>
@@ -14148,7 +14148,7 @@
         <v>15.5962962962963</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="15.75">
       <c r="A12" s="1">
         <v>13075020</v>
       </c>
@@ -14262,7 +14262,7 @@
         <v>17.520689655172415</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="15.75">
       <c r="A13" s="1">
         <v>12045020</v>
       </c>
@@ -14374,7 +14374,7 @@
       </c>
       <c r="AK13" s="8"/>
     </row>
-    <row r="14" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="15.75">
       <c r="A14" s="1">
         <v>13075010</v>
       </c>
@@ -14488,7 +14488,7 @@
         <v>15.077777777777776</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="15.75">
       <c r="A15" s="1">
         <v>13030010</v>
       </c>
@@ -14602,7 +14602,7 @@
         <v>22.771999999999998</v>
       </c>
     </row>
-    <row r="17" spans="4:35" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:35" ht="15.75">
       <c r="D17" s="20" t="s">
         <v>31</v>
       </c>
@@ -14792,22 +14792,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2476E830-F9B1-4C5E-B87D-BCCDD21D9D78}">
   <dimension ref="A2:AK17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="21" width="5.85546875" style="27" customWidth="1"/>
-    <col min="22" max="22" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.85546875" customWidth="1"/>
-    <col min="24" max="26" width="4.5703125" customWidth="1"/>
-    <col min="27" max="27" width="5.85546875" customWidth="1"/>
-    <col min="28" max="28" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="35" width="4.5703125" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="4" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="21" width="5.875" style="27" customWidth="1"/>
+    <col min="22" max="22" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.875" customWidth="1"/>
+    <col min="24" max="26" width="4.625" customWidth="1"/>
+    <col min="27" max="27" width="5.875" customWidth="1"/>
+    <col min="28" max="28" width="5.75" bestFit="1" customWidth="1"/>
+    <col min="29" max="35" width="4.625" customWidth="1"/>
     <col min="36" max="36" width="16" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.42578125" customWidth="1"/>
+    <col min="37" max="37" width="14.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" ht="15.75">
       <c r="A2" s="17" t="s">
         <v>26</v>
       </c>
@@ -14920,7 +14920,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" ht="15.75">
       <c r="A3" s="1">
         <v>13035501</v>
       </c>
@@ -15028,7 +15028,7 @@
         <v>11.108333333333333</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" ht="15.75">
       <c r="A4" s="1">
         <v>25025170</v>
       </c>
@@ -15136,7 +15136,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" ht="15.75">
       <c r="A5" s="1">
         <v>25020140</v>
       </c>
@@ -15244,7 +15244,7 @@
         <v>26.736666666666668</v>
       </c>
     </row>
-    <row r="6" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="15.75">
       <c r="A6" s="1">
         <v>25025160</v>
       </c>
@@ -15352,7 +15352,7 @@
         <v>24.500000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="15.75">
       <c r="A7" s="1">
         <v>25025190</v>
       </c>
@@ -15460,7 +15460,7 @@
         <v>12.814285714285713</v>
       </c>
     </row>
-    <row r="8" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="15.75">
       <c r="A8" s="1">
         <v>25020470</v>
       </c>
@@ -15568,7 +15568,7 @@
         <v>21.427586206896549</v>
       </c>
     </row>
-    <row r="9" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="15.75">
       <c r="A9" s="1">
         <v>25020700</v>
       </c>
@@ -15668,7 +15668,7 @@
         <v>19.775862068965512</v>
       </c>
     </row>
-    <row r="10" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="15.75">
       <c r="A10" s="1">
         <v>13015040</v>
       </c>
@@ -15774,7 +15774,7 @@
       </c>
       <c r="AK10" s="8"/>
     </row>
-    <row r="11" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="15.75">
       <c r="A11" s="1">
         <v>13085010</v>
       </c>
@@ -15880,7 +15880,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="15.75">
       <c r="A12" s="1">
         <v>13075020</v>
       </c>
@@ -15988,7 +15988,7 @@
         <v>18.257142857142856</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="15.75">
       <c r="A13" s="1">
         <v>12045020</v>
       </c>
@@ -16090,7 +16090,7 @@
       </c>
       <c r="AK13" s="8"/>
     </row>
-    <row r="14" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="15.75">
       <c r="A14" s="1">
         <v>13075010</v>
       </c>
@@ -16196,7 +16196,7 @@
         <v>13.462068965517243</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="15.75">
       <c r="A15" s="1">
         <v>13030010</v>
       </c>
@@ -16304,7 +16304,7 @@
         <v>19.926923076923078</v>
       </c>
     </row>
-    <row r="17" spans="4:35" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:35" ht="15.75">
       <c r="D17" s="20" t="s">
         <v>31</v>
       </c>
@@ -16447,22 +16447,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{794DFC6B-8D5A-4452-84E9-AF1FA7EDAD6A}">
   <dimension ref="A2:AK17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="21" width="5.85546875" style="27" customWidth="1"/>
-    <col min="22" max="22" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.85546875" customWidth="1"/>
-    <col min="24" max="24" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="4.5703125" customWidth="1"/>
-    <col min="27" max="30" width="5.7109375" customWidth="1"/>
-    <col min="31" max="35" width="4.5703125" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="4" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="21" width="5.875" style="27" customWidth="1"/>
+    <col min="22" max="22" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.875" customWidth="1"/>
+    <col min="24" max="24" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="4.625" customWidth="1"/>
+    <col min="27" max="30" width="5.75" customWidth="1"/>
+    <col min="31" max="35" width="4.625" customWidth="1"/>
     <col min="36" max="36" width="16" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.42578125" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="14.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" ht="15.75">
       <c r="A2" s="17" t="s">
         <v>26</v>
       </c>
@@ -16575,7 +16575,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" ht="15.75">
       <c r="A3" s="1">
         <v>13035501</v>
       </c>
@@ -16687,7 +16687,7 @@
         <v>27.817857142857147</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" ht="15.75">
       <c r="A4" s="1">
         <v>25025170</v>
       </c>
@@ -16799,7 +16799,7 @@
         <v>47.628571428571419</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" ht="15.75">
       <c r="A5" s="1">
         <v>25020140</v>
       </c>
@@ -16911,7 +16911,7 @@
         <v>40.986206896551728</v>
       </c>
     </row>
-    <row r="6" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="15.75">
       <c r="A6" s="1">
         <v>25025160</v>
       </c>
@@ -17023,7 +17023,7 @@
         <v>88.719230769230762</v>
       </c>
     </row>
-    <row r="7" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="15.75">
       <c r="A7" s="1">
         <v>25025190</v>
       </c>
@@ -17135,7 +17135,7 @@
         <v>48.014814814814812</v>
       </c>
     </row>
-    <row r="8" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="15.75">
       <c r="A8" s="1">
         <v>25020470</v>
       </c>
@@ -17247,7 +17247,7 @@
         <v>47.275862068965516</v>
       </c>
     </row>
-    <row r="9" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="15.75">
       <c r="A9" s="1">
         <v>25020700</v>
       </c>
@@ -17299,7 +17299,7 @@
         <v>65.482758620689651</v>
       </c>
     </row>
-    <row r="10" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="15.75">
       <c r="A10" s="1">
         <v>13015040</v>
       </c>
@@ -17409,7 +17409,7 @@
       </c>
       <c r="AK10" s="8"/>
     </row>
-    <row r="11" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="15.75">
       <c r="A11" s="1">
         <v>13085010</v>
       </c>
@@ -17461,7 +17461,7 @@
         <v>19.188461538461539</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="15.75">
       <c r="A12" s="1">
         <v>13075020</v>
       </c>
@@ -17573,7 +17573,7 @@
         <v>34.724137931034484</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="15.75">
       <c r="A13" s="1">
         <v>12045020</v>
       </c>
@@ -17683,7 +17683,7 @@
       </c>
       <c r="AK13" s="8"/>
     </row>
-    <row r="14" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="15.75">
       <c r="A14" s="1">
         <v>13075010</v>
       </c>
@@ -17795,7 +17795,7 @@
         <v>36.1</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="15.75">
       <c r="A15" s="1">
         <v>13030010</v>
       </c>
@@ -17907,7 +17907,7 @@
         <v>60.46</v>
       </c>
     </row>
-    <row r="17" spans="4:35" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:35" ht="15">
       <c r="D17" s="20" t="s">
         <v>31</v>
       </c>
@@ -18050,24 +18050,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9B00C4-7439-424E-B84E-4F748B6DBCED}">
   <dimension ref="A2:AK19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.42578125" customWidth="1"/>
-    <col min="5" max="21" width="5.85546875" style="27" customWidth="1"/>
-    <col min="22" max="22" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.85546875" customWidth="1"/>
-    <col min="24" max="24" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="4.5703125" customWidth="1"/>
-    <col min="27" max="30" width="5.7109375" customWidth="1"/>
-    <col min="31" max="35" width="4.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.125" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.375" customWidth="1"/>
+    <col min="5" max="21" width="5.875" style="27" customWidth="1"/>
+    <col min="22" max="22" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.875" customWidth="1"/>
+    <col min="24" max="24" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="4.625" customWidth="1"/>
+    <col min="27" max="30" width="5.75" customWidth="1"/>
+    <col min="31" max="35" width="4.625" customWidth="1"/>
     <col min="36" max="36" width="16" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.42578125" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="14.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" ht="15.75">
       <c r="A2" s="17" t="s">
         <v>26</v>
       </c>
@@ -18180,7 +18180,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" ht="15.75">
       <c r="A3" s="1">
         <v>13035501</v>
       </c>
@@ -18294,7 +18294,7 @@
         <v>27.817857142857147</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" ht="15.75">
       <c r="A4" s="1">
         <v>25020470</v>
       </c>
@@ -18408,7 +18408,7 @@
         <v>47.628571428571419</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" ht="15.75">
       <c r="A5" s="1">
         <v>25025160</v>
       </c>
@@ -18522,7 +18522,7 @@
         <v>40.986206896551728</v>
       </c>
     </row>
-    <row r="6" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="15.75">
       <c r="A6" s="1">
         <v>13015040</v>
       </c>
@@ -18636,7 +18636,7 @@
         <v>88.719230769230762</v>
       </c>
     </row>
-    <row r="7" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="15.75">
       <c r="A7" s="1">
         <v>13085010</v>
       </c>
@@ -18688,7 +18688,7 @@
         <v>48.014814814814812</v>
       </c>
     </row>
-    <row r="8" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="15.75">
       <c r="A8" s="1">
         <v>25020700</v>
       </c>
@@ -18740,7 +18740,7 @@
         <v>47.275862068965516</v>
       </c>
     </row>
-    <row r="9" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="15.75">
       <c r="A9" s="1">
         <v>13030010</v>
       </c>
@@ -18854,7 +18854,7 @@
         <v>65.482758620689651</v>
       </c>
     </row>
-    <row r="10" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="15.75">
       <c r="A10" s="1">
         <v>25025190</v>
       </c>
@@ -18966,7 +18966,7 @@
       </c>
       <c r="AK10" s="30"/>
     </row>
-    <row r="11" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="15.75">
       <c r="A11" s="1">
         <v>13075020</v>
       </c>
@@ -19078,7 +19078,7 @@
         <v>19.188461538461539</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="15.75">
       <c r="A12" s="1">
         <v>12045020</v>
       </c>
@@ -19188,7 +19188,7 @@
         <v>34.724137931034484</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="15.75">
       <c r="A13" s="1">
         <v>25025170</v>
       </c>
@@ -19300,7 +19300,7 @@
       </c>
       <c r="AK13" s="30"/>
     </row>
-    <row r="14" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="15.75">
       <c r="A14" s="1">
         <v>13075010</v>
       </c>
@@ -19412,7 +19412,7 @@
         <v>36.1</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="15.75">
       <c r="A15" s="1">
         <v>25020140</v>
       </c>
@@ -19526,7 +19526,7 @@
         <v>60.46</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" ht="15.75">
       <c r="A16" s="1">
         <v>13057010</v>
       </c>
@@ -19579,7 +19579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="15.75">
       <c r="A17" s="1">
         <v>13085030</v>
       </c>
@@ -19632,7 +19632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="15.75">
       <c r="D19" s="33" t="s">
         <v>31</v>
       </c>
@@ -19775,25 +19775,25 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A42E600-7B4A-4F11-AF73-65461A008112}">
   <dimension ref="A2:AK19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.42578125" customWidth="1"/>
-    <col min="5" max="21" width="5.85546875" style="27" customWidth="1"/>
-    <col min="22" max="22" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.85546875" customWidth="1"/>
-    <col min="24" max="24" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="4.5703125" customWidth="1"/>
-    <col min="26" max="26" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="30" width="5.7109375" customWidth="1"/>
-    <col min="31" max="35" width="4.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.125" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.375" customWidth="1"/>
+    <col min="5" max="21" width="5.875" style="27" customWidth="1"/>
+    <col min="22" max="22" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.875" customWidth="1"/>
+    <col min="24" max="24" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="4.625" customWidth="1"/>
+    <col min="26" max="26" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="27" max="30" width="5.75" customWidth="1"/>
+    <col min="31" max="35" width="4.625" customWidth="1"/>
     <col min="36" max="36" width="16" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.42578125" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="14.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" ht="15.75">
       <c r="A2" s="17" t="s">
         <v>26</v>
       </c>
@@ -19906,7 +19906,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" ht="15.75">
       <c r="A3" s="1">
         <v>13035501</v>
       </c>
@@ -19964,7 +19964,9 @@
       <c r="S3" s="25">
         <v>0</v>
       </c>
-      <c r="T3" s="25"/>
+      <c r="T3" s="25">
+        <v>0</v>
+      </c>
       <c r="U3" s="25"/>
       <c r="V3" s="25"/>
       <c r="W3" s="25"/>
@@ -19988,7 +19990,7 @@
         <v>27.817857142857147</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" ht="15.75">
       <c r="A4" s="1">
         <v>25020470</v>
       </c>
@@ -20070,7 +20072,7 @@
         <v>47.628571428571419</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" ht="15.75">
       <c r="A5" s="1">
         <v>25025160</v>
       </c>
@@ -20128,7 +20130,9 @@
       <c r="S5" s="25">
         <v>0</v>
       </c>
-      <c r="T5" s="25"/>
+      <c r="T5" s="25">
+        <v>0</v>
+      </c>
       <c r="U5" s="25"/>
       <c r="V5" s="25"/>
       <c r="W5" s="25"/>
@@ -20152,7 +20156,7 @@
         <v>40.986206896551728</v>
       </c>
     </row>
-    <row r="6" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="15.75">
       <c r="A6" s="1">
         <v>13015040</v>
       </c>
@@ -20210,7 +20214,9 @@
       <c r="S6" s="25">
         <v>0</v>
       </c>
-      <c r="T6" s="25"/>
+      <c r="T6" s="25">
+        <v>0</v>
+      </c>
       <c r="U6" s="25"/>
       <c r="V6" s="25"/>
       <c r="W6" s="25"/>
@@ -20234,7 +20240,7 @@
         <v>88.719230769230762</v>
       </c>
     </row>
-    <row r="7" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="15.75">
       <c r="A7" s="1">
         <v>13085010</v>
       </c>
@@ -20286,7 +20292,7 @@
         <v>48.014814814814812</v>
       </c>
     </row>
-    <row r="8" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="15.75">
       <c r="A8" s="1">
         <v>25020700</v>
       </c>
@@ -20338,7 +20344,7 @@
         <v>47.275862068965516</v>
       </c>
     </row>
-    <row r="9" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="15.75">
       <c r="A9" s="1">
         <v>13030010</v>
       </c>
@@ -20396,7 +20402,9 @@
       <c r="S9" s="25">
         <v>0</v>
       </c>
-      <c r="T9" s="25"/>
+      <c r="T9" s="25">
+        <v>0</v>
+      </c>
       <c r="U9" s="25"/>
       <c r="V9" s="25"/>
       <c r="W9" s="25"/>
@@ -20420,7 +20428,7 @@
         <v>65.482758620689651</v>
       </c>
     </row>
-    <row r="10" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="15.75">
       <c r="A10" s="1">
         <v>25025190</v>
       </c>
@@ -20498,7 +20506,7 @@
       </c>
       <c r="AK10" s="30"/>
     </row>
-    <row r="11" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="15.75">
       <c r="A11" s="1">
         <v>13075020</v>
       </c>
@@ -20556,7 +20564,9 @@
       <c r="S11" s="25">
         <v>0</v>
       </c>
-      <c r="T11" s="25"/>
+      <c r="T11" s="25">
+        <v>0</v>
+      </c>
       <c r="U11" s="25"/>
       <c r="V11" s="25"/>
       <c r="W11" s="25"/>
@@ -20580,7 +20590,7 @@
         <v>19.188461538461539</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="15.75">
       <c r="A12" s="1">
         <v>12045020</v>
       </c>
@@ -20636,7 +20646,9 @@
       <c r="S12" s="25">
         <v>0</v>
       </c>
-      <c r="T12" s="25"/>
+      <c r="T12" s="25">
+        <v>0</v>
+      </c>
       <c r="U12" s="25"/>
       <c r="V12" s="25"/>
       <c r="W12" s="25"/>
@@ -20660,7 +20672,7 @@
         <v>34.724137931034484</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="15.75">
       <c r="A13" s="1">
         <v>25025170</v>
       </c>
@@ -20718,7 +20730,9 @@
       <c r="S13" s="25">
         <v>0</v>
       </c>
-      <c r="T13" s="25"/>
+      <c r="T13" s="25">
+        <v>0</v>
+      </c>
       <c r="U13" s="25"/>
       <c r="V13" s="25"/>
       <c r="W13" s="25"/>
@@ -20740,7 +20754,7 @@
       </c>
       <c r="AK13" s="30"/>
     </row>
-    <row r="14" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="15.75">
       <c r="A14" s="1">
         <v>13075010</v>
       </c>
@@ -20798,7 +20812,9 @@
       <c r="S14" s="25">
         <v>0</v>
       </c>
-      <c r="T14" s="25"/>
+      <c r="T14" s="25">
+        <v>0</v>
+      </c>
       <c r="U14" s="25"/>
       <c r="V14" s="25"/>
       <c r="W14" s="25"/>
@@ -20822,7 +20838,7 @@
         <v>36.1</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="15.75">
       <c r="A15" s="1">
         <v>25020140</v>
       </c>
@@ -20880,7 +20896,9 @@
       <c r="S15" s="25">
         <v>0</v>
       </c>
-      <c r="T15" s="25"/>
+      <c r="T15" s="25">
+        <v>0</v>
+      </c>
       <c r="U15" s="25"/>
       <c r="V15" s="25"/>
       <c r="W15" s="25"/>
@@ -20904,7 +20922,7 @@
         <v>60.46</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" ht="15.75">
       <c r="A16" s="1">
         <v>13057010</v>
       </c>
@@ -20953,7 +20971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="15.75">
       <c r="A17" s="1">
         <v>13085030</v>
       </c>
@@ -21002,7 +21020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="15.75">
       <c r="D19" s="33" t="s">
         <v>31</v>
       </c>
@@ -21068,7 +21086,7 @@
       </c>
       <c r="T19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U19" s="26">
         <f t="shared" si="1"/>

</xml_diff>